<commit_message>
fixed: consultas flujo de leads
</commit_message>
<xml_diff>
--- a/data/estad_portales/Rendimiento_período-p1.xlsx
+++ b/data/estad_portales/Rendimiento_período-p1.xlsx
@@ -427,25 +427,25 @@
     </row>
     <row r="2" ht="17" customHeight="1">
       <c r="A2" s="2" t="str">
-        <v>04/09/2026</v>
+        <v>11/09/2026</v>
       </c>
       <c r="B2" s="2">
-        <v>20762</v>
+        <v>18617</v>
       </c>
       <c r="C2" s="2">
-        <v>1054</v>
+        <v>1143</v>
       </c>
       <c r="D2" s="2">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="E2" s="2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F2" s="2">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H2" s="2" t="str">
         <v/>
@@ -453,25 +453,25 @@
     </row>
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="2" t="str">
-        <v>05/09/2026</v>
+        <v>12/09/2026</v>
       </c>
       <c r="B3" s="2">
-        <v>20443</v>
+        <v>19319</v>
       </c>
       <c r="C3" s="2">
-        <v>1022</v>
+        <v>1137</v>
       </c>
       <c r="D3" s="2">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="E3" s="2">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="F3" s="2">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G3" s="2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H3" s="2" t="str">
         <v/>
@@ -479,25 +479,25 @@
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="A4" s="2" t="str">
-        <v>06/09/2026</v>
+        <v>13/09/2026</v>
       </c>
       <c r="B4" s="2">
-        <v>22882</v>
+        <v>21432</v>
       </c>
       <c r="C4" s="2">
-        <v>1032</v>
+        <v>1190</v>
       </c>
       <c r="D4" s="2">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="E4" s="2">
         <v>10</v>
       </c>
       <c r="F4" s="2">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="G4" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H4" s="2" t="str">
         <v/>
@@ -505,25 +505,25 @@
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="2" t="str">
-        <v>07/09/2026</v>
+        <v>14/09/2026</v>
       </c>
       <c r="B5" s="2">
-        <v>23242</v>
+        <v>21536</v>
       </c>
       <c r="C5" s="2">
-        <v>1296</v>
+        <v>1249</v>
       </c>
       <c r="D5" s="2">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E5" s="2">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F5" s="2">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G5" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H5" s="2" t="str">
         <v/>
@@ -531,25 +531,25 @@
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="2" t="str">
-        <v>08/09/2026</v>
+        <v>15/09/2026</v>
       </c>
       <c r="B6" s="2">
-        <v>24407</v>
+        <v>17618</v>
       </c>
       <c r="C6" s="2">
-        <v>1270</v>
+        <v>1090</v>
       </c>
       <c r="D6" s="2">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E6" s="2">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F6" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G6" s="2">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H6" s="2" t="str">
         <v/>
@@ -557,25 +557,25 @@
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="2" t="str">
-        <v>09/09/2026</v>
+        <v>16/09/2026</v>
       </c>
       <c r="B7" s="2">
-        <v>20996</v>
+        <v>23237</v>
       </c>
       <c r="C7" s="2">
-        <v>1233</v>
+        <v>1429</v>
       </c>
       <c r="D7" s="2">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="E7" s="2">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="F7" s="2">
         <v>11</v>
       </c>
       <c r="G7" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H7" s="2" t="str">
         <v/>
@@ -583,25 +583,25 @@
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="2" t="str">
-        <v>10/09/2026</v>
+        <v>17/09/2026</v>
       </c>
       <c r="B8" s="2">
-        <v>19769</v>
+        <v>26024</v>
       </c>
       <c r="C8" s="2">
-        <v>1161</v>
+        <v>1706</v>
       </c>
       <c r="D8" s="2">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="E8" s="2">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F8" s="2">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="G8" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H8" s="2" t="str">
         <v/>

</xml_diff>